<commit_message>
added checks in time
</commit_message>
<xml_diff>
--- a/src/main/resources/file/Transactional.xlsx
+++ b/src/main/resources/file/Transactional.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chinb./"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ca/Developer/Projects/jtgm-excel-processor/src/main/resources/file/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5394DEF-1537-4C46-9643-624375917A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED96CC7A-D7C4-E44A-BFD1-DC564A1D5CAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="500" windowWidth="28040" windowHeight="16480" xr2:uid="{0D444C09-E85E-734F-B86B-83E709D6E31A}"/>
+    <workbookView xWindow="760" yWindow="660" windowWidth="28040" windowHeight="16480" xr2:uid="{0D444C09-E85E-734F-B86B-83E709D6E31A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Date</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>Attendee ID</t>
+  </si>
+  <si>
+    <t>Time</t>
   </si>
 </sst>
 </file>
@@ -440,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{782CE1E8-6C29-4F42-8DF1-B0C7F03C0560}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" style="1" bestFit="1" customWidth="1" collapsed="1"/>
@@ -451,10 +454,10 @@
     <col min="6" max="6" width="14.83203125" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="7" max="7" width="9.1640625" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="8" max="8" width="25.1640625" customWidth="1" collapsed="1"/>
-    <col min="9" max="9" width="19.83203125" customWidth="1" collapsed="1"/>
+    <col min="9" max="10" width="19.83203125" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -481,6 +484,9 @@
       </c>
       <c r="I1" s="3" t="s">
         <v>6</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>